<commit_message>
Initial Playwright Cucumber framework
</commit_message>
<xml_diff>
--- a/src/testdata/data.xlsx
+++ b/src/testdata/data.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Course\Playwright_typescript\Playwright_April26\Playwright_Cucumber_Framework\src\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Playwright_Automation\Playwright_Cucumber_Framework\src\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D555DFEF-87F1-4FA5-9D64-ED74EA1CE674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{3DF1D48F-7064-43B5-B4B0-DC020BA99D61}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="21792" windowHeight="12972"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>TCName</t>
   </si>
@@ -65,13 +64,40 @@
   </si>
   <si>
     <t>SpaceX</t>
+  </si>
+  <si>
+    <t>verify_create_account_with_mandatory_fields_TC05</t>
+  </si>
+  <si>
+    <t>accountname</t>
+  </si>
+  <si>
+    <t>Employees</t>
+  </si>
+  <si>
+    <t>ABC Software</t>
+  </si>
+  <si>
+    <t>verify_create_contact_with_mandatory_fields_TC06</t>
+  </si>
+  <si>
+    <t>Miraje</t>
+  </si>
+  <si>
+    <t>Shivaji</t>
+  </si>
+  <si>
+    <t>first</t>
+  </si>
+  <si>
+    <t>Last</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -409,7 +435,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -539,6 +565,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -584,10 +621,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -962,18 +1001,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B858FA1-F6C4-4A31-BB4E-D8ACA92F9760}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="48.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="48.296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.8984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.3984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" ht="17.399999999999999">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -992,8 +1031,20 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" ht="17.399999999999999">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1005,7 +1056,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" ht="17.399999999999999">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -1019,7 +1070,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" ht="17.399999999999999">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -1033,7 +1084,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" ht="17.399999999999999">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1051,7 +1102,42 @@
         <v>14</v>
       </c>
     </row>
+    <row r="6" spans="1:10" ht="17.399999999999999">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="17.399999999999999">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>